<commit_message>
update excel merge logic
</commit_message>
<xml_diff>
--- a/data/1_2.xlsx
+++ b/data/1_2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="27">
   <si>
     <r>
       <t>Код и наименова ние ка</t>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Итого по факультету ФИТР</t>
+  </si>
+  <si>
+    <t>ИТОГО</t>
   </si>
 </sst>
 </file>
@@ -157,7 +160,7 @@
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +182,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0B0"/>
       </patternFill>
     </fill>
   </fills>
@@ -235,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -261,6 +269,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -270,6 +279,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -609,7 +619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -885,106 +895,106 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" ht="19.5" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="4" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="E10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="19.5" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="H11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="3">
-        <v>10701125</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="3">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="M11" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="3">
-        <v>10701225</v>
-      </c>
-      <c r="D12" s="9" t="s">
+        <v>10701125</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>15</v>
@@ -1005,7 +1015,7 @@
         <v>15</v>
       </c>
       <c r="M12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1016,16 +1026,16 @@
         <v>23</v>
       </c>
       <c r="C13" s="3">
-        <v>10701325</v>
-      </c>
-      <c r="D13" s="9" t="s">
+        <v>10701225</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>15</v>
+      <c r="F13" s="3">
+        <v>2</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>15</v>
@@ -1045,8 +1055,8 @@
       <c r="L13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M13" s="3" t="s">
-        <v>15</v>
+      <c r="M13" s="3">
+        <v>2</v>
       </c>
     </row>
     <row r="14" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1057,16 +1067,16 @@
         <v>23</v>
       </c>
       <c r="C14" s="3">
-        <v>10702325</v>
-      </c>
-      <c r="D14" s="9" t="s">
+        <v>10701325</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F14" s="3">
-        <v>2</v>
+      <c r="F14" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>15</v>
@@ -1086,11 +1096,11 @@
       <c r="L14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M14" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" ht="38.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M14" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
@@ -1098,16 +1108,16 @@
         <v>23</v>
       </c>
       <c r="C15" s="3">
-        <v>10702425</v>
-      </c>
-      <c r="D15" s="9" t="s">
+        <v>10702325</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>15</v>
@@ -1128,10 +1138,10 @@
         <v>15</v>
       </c>
       <c r="M15" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="38.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>24</v>
       </c>
@@ -1139,9 +1149,9 @@
         <v>23</v>
       </c>
       <c r="C16" s="3">
-        <v>10705125</v>
-      </c>
-      <c r="D16" s="9" t="s">
+        <v>10702425</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -1180,16 +1190,16 @@
         <v>23</v>
       </c>
       <c r="C17" s="3">
-        <v>10705225</v>
-      </c>
-      <c r="D17" s="9" t="s">
+        <v>10705125</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>15</v>
+      <c r="F17" s="3">
+        <v>1</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>15</v>
@@ -1209,8 +1219,8 @@
       <c r="L17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M17" s="3" t="s">
-        <v>15</v>
+      <c r="M17" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="18" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1221,16 +1231,16 @@
         <v>23</v>
       </c>
       <c r="C18" s="3">
-        <v>10703125</v>
-      </c>
-      <c r="D18" s="9" t="s">
+        <v>10705225</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="3">
-        <v>1</v>
+      <c r="F18" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>15</v>
@@ -1250,8 +1260,8 @@
       <c r="L18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M18" s="3">
-        <v>1</v>
+      <c r="M18" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="19" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1262,16 +1272,16 @@
         <v>23</v>
       </c>
       <c r="C19" s="3">
-        <v>10703225</v>
-      </c>
-      <c r="D19" s="9" t="s">
+        <v>10703125</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>15</v>
@@ -1292,7 +1302,7 @@
         <v>15</v>
       </c>
       <c r="M19" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1303,16 +1313,16 @@
         <v>23</v>
       </c>
       <c r="C20" s="3">
-        <v>10706125</v>
-      </c>
-      <c r="D20" s="9" t="s">
+        <v>10703225</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>15</v>
@@ -1333,7 +1343,7 @@
         <v>15</v>
       </c>
       <c r="M20" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1344,74 +1354,156 @@
         <v>23</v>
       </c>
       <c r="C21" s="3">
+        <v>10706125</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="3">
+        <v>3</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M21" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" ht="51" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="3">
         <v>10701425</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="M21" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="D22" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="6">
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="6">
         <v>13</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="K22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L22" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="M22" s="6">
+      <c r="G23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="M23" s="6">
         <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="M24" s="13">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1453,7 +1545,7 @@
     <mergeCell ref="K7:K8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="M7:M8"/>
-    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A23:C23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
full info final row
</commit_message>
<xml_diff>
--- a/data/1_2.xlsx
+++ b/data/1_2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="27">
   <si>
     <r>
       <t>Код и наименова ние ка</t>
@@ -1481,11 +1481,11 @@
       <c r="E24" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="13" t="s">
-        <v>15</v>
+      <c r="F24" s="13">
+        <v>13</v>
+      </c>
+      <c r="G24" s="13">
+        <v>4</v>
       </c>
       <c r="H24" s="13" t="s">
         <v>15</v>

</xml_diff>